<commit_message>
Criando tabela com Indice
</commit_message>
<xml_diff>
--- a/folha_pagamento.xlsx
+++ b/folha_pagamento.xlsx
@@ -425,75 +425,87 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>NOME</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>IDADE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>SALARIO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Matheus</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>19</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Otavio</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>18</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>3000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Luiz</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>19</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Gabriel</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>20</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>